<commit_message>
atualizando excel com refinamento das historias
</commit_message>
<xml_diff>
--- a/Close Care/(excel) Ordem de prioridade.xlsx
+++ b/Close Care/(excel) Ordem de prioridade.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\uniflgoncalves\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\uniflgoncalves\Documents\GitHub\CloseCare-GEST.PROJ.SOFT\Close Care\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F45F3922-739E-4454-8EFD-12969A608F1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FECA6CBB-A5D7-4880-B9AE-27675E53EA1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4B4DFAF-313B-4775-A4C5-2B6A73696C89}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="38">
   <si>
     <t>ID</t>
   </si>
@@ -95,36 +95,12 @@
     <t>Como paciente, quero agendar um exame para realizá-lo em uma data conveniente.</t>
   </si>
   <si>
-    <t>Como profissional de saúde, quero solicitar uma consulta para um paciente para garantir a continuidade do tratamento.</t>
-  </si>
-  <si>
     <t>Should</t>
   </si>
   <si>
-    <t>Como profissional de saúde, quero solicitar um exame para um paciente para apoiar o diagnóstico.</t>
-  </si>
-  <si>
     <t>Como paciente ou profissional, quero visualizar as consultas cadastradas para acompanhar os atendimentos.</t>
   </si>
   <si>
-    <t>Como paciente ou profissional, quero visualizar os exames cadastrados para acompanhar as solicitações e agendamentos.</t>
-  </si>
-  <si>
-    <t>Como paciente ou profissional, quero remarcar uma consulta para adequar o atendimento à disponibilidade.</t>
-  </si>
-  <si>
-    <t>Como paciente ou profissional, quero remarcar um exame para ajustar sua realização.</t>
-  </si>
-  <si>
-    <t>Como paciente ou profissional, quero cancelar uma consulta para liberar o horário quando não puder comparecer.</t>
-  </si>
-  <si>
-    <t>Como paciente ou profissional, quero cancelar um exame para liberar o horário reservado.</t>
-  </si>
-  <si>
-    <t>Como profissional de saúde, quero definir datas e horários disponíveis para que pacientes possam realizar agendamentos.</t>
-  </si>
-  <si>
     <t>HU12</t>
   </si>
   <si>
@@ -138,6 +114,57 @@
   </si>
   <si>
     <t>x</t>
+  </si>
+  <si>
+    <t>Como paciente com mobilidade reduzida ou idoso, quero agendar uma consulta domiciliar selecionando o tipo de profissional, a data, o horário e 
+o meu endereço cadastrado para receber atendimento médico em casa com conforto, sem a necessidade de deslocamento.</t>
+  </si>
+  <si>
+    <t>Como paciente com mobilidade reduzida ou idoso, quero agendar a realização de um exame domiciliar informando a data e horário conveniente 
+com o profissional desejado para realizar exames diagnósticos sem sair de casa e sem enfrentar barreiras de acessibilidade.</t>
+  </si>
+  <si>
+    <t>Como profissional de saúde, quero solicitar/encaminhar uma consulta de retorno ou especialidade para um paciente cadastrado para garantir 
+a continuidade do tratamento e o acompanhamento preventivo do paciente</t>
+  </si>
+  <si>
+    <t>Como profissional de saúde, quero solicitar um pedido de exame domiciliar vinculando o tipo de exame e orientações 
+de preparo ao paciente para orientar a equipe ou mesmo o profissional encarregado e embasar o diagnóstico clínico do paciente.</t>
+  </si>
+  <si>
+    <t>Como paciente ou profissional de saúde, quero visualizar a lista de consultas cadastradas para acompanhar os atendimentos agendados.</t>
+  </si>
+  <si>
+    <t>Como paciente ou profissional de saúde, quero consultar a lista de exames cadastrados para acompanhar as solicitações e agendamentos
+para verificar os laudos disponibilizados.</t>
+  </si>
+  <si>
+    <t>Como paciente ou profissional de saúde, quero alterar a data e o horário de uma consulta domiciliar já agendada por conta de imprevistos 
+de agenda de uma ou ambas as partes.</t>
+  </si>
+  <si>
+    <t>Como paciente ou profissional de saúde, quero remarcar a data e/ou horário de um exame ja agendado por conta de imprevistos 
+de agenda de uma ou ambas as partes.</t>
+  </si>
+  <si>
+    <t>Como paciente ou profissional de saúde, quero cancelar uma consulta domiciliar previamente confirmada por conta de 
+imprevistos na agenda de uma ou ambas as partes.</t>
+  </si>
+  <si>
+    <t>Como paciente ou profissional de saúde, quero cancelar um exame domiciliar previamente confirmada por conta de 
+imprevistos na agenda de uma ou ambas as partes.</t>
+  </si>
+  <si>
+    <t>Como profissional de saúde, quero cadastrar meus horários de atendimento, especialidade e raio de distância que aceito percorrer para visitas
+Para restringir e permitir que apenas pacientes localizados na minha área designada consigam agendar consultas.</t>
+  </si>
+  <si>
+    <t>Como paciente com falta de mobilidade ou profissional, quero cadastrar uma conta no aplicativo inserindo meus dados para acessar os serviços 
+de atendimento domiciliar conforme o meu tipo de conta.</t>
+  </si>
+  <si>
+    <t>Como paciente com falta de mobilidade ou profissional, quero realizar login digitando minhas credenciais no aplicativo 
+para acessar minha conta e utilizar as funcionalidades disponíveis da plataforma.</t>
   </si>
 </sst>
 </file>
@@ -197,7 +224,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -217,16 +244,22 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="5">
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -256,8 +289,8 @@
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{985DA469-90E4-4E24-8BE5-72DD8AC4D4B7}" name="Prioridade" totalsRowLabel="Total" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{8CF543ED-69A6-4089-B1C8-916B531B30CB}" name="ID" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{DF14E0CF-8CC5-458E-9DBC-9D271FF5D8AF}" name="Historia" dataDxfId="1"/>
-    <tableColumn id="9" xr3:uid="{E588BD5A-7EF6-439C-8B85-7F5F2AAF23CB}" name="MosCow" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{DF14E0CF-8CC5-458E-9DBC-9D271FF5D8AF}" name="Historia" dataDxfId="0"/>
+    <tableColumn id="9" xr3:uid="{E588BD5A-7EF6-439C-8B85-7F5F2AAF23CB}" name="MosCow" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="0" showRowStripes="1" showColumnStripes="1"/>
 </table>
@@ -604,87 +637,87 @@
       </c>
       <c r="F2" s="1"/>
     </row>
-    <row r="3" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:6" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="5">
         <v>1</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>31</v>
+        <v>20</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>36</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>16</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="4" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="5">
         <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>30</v>
+        <v>21</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>37</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>16</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="5">
         <v>3</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>27</v>
+      <c r="D5" s="8" t="s">
+        <v>35</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>16</v>
       </c>
       <c r="F5" s="1"/>
     </row>
-    <row r="6" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:6" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="5">
         <v>4</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>13</v>
+      <c r="D6" s="8" t="s">
+        <v>25</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>16</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="5">
         <v>5</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>17</v>
+      <c r="D7" s="8" t="s">
+        <v>26</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>16</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -694,118 +727,118 @@
       <c r="C8" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>21</v>
+      <c r="D8" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>16</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="9" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="5">
         <v>7</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>22</v>
+      <c r="D9" s="8" t="s">
+        <v>30</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>16</v>
       </c>
       <c r="F9" s="1"/>
     </row>
-    <row r="10" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:6" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="5">
         <v>8</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>25</v>
+      <c r="D10" s="8" t="s">
+        <v>33</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>16</v>
       </c>
       <c r="F10" s="1"/>
     </row>
-    <row r="11" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:6" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="5">
         <v>9</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>26</v>
+      <c r="D11" s="8" t="s">
+        <v>34</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>16</v>
       </c>
       <c r="F11" s="1"/>
     </row>
-    <row r="12" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:6" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="5">
         <v>10</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E12" s="4" t="s">
-        <v>19</v>
-      </c>
       <c r="F12" s="1"/>
     </row>
-    <row r="13" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:6" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="5">
         <v>11</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>20</v>
+      <c r="D13" s="8" t="s">
+        <v>28</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F13" s="1"/>
     </row>
-    <row r="14" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:6" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="5">
         <v>12</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>23</v>
+      <c r="D14" s="8" t="s">
+        <v>31</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F14" s="1"/>
     </row>
-    <row r="15" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:6" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="5">
         <v>13</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>24</v>
+      <c r="D15" s="8" t="s">
+        <v>32</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F15" s="1"/>
     </row>
@@ -829,16 +862,16 @@
         <v>1</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>16</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
     </row>
     <row r="37" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -846,16 +879,16 @@
         <v>2</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="E37" s="3" t="s">
         <v>16</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
     </row>
     <row r="38" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -872,7 +905,7 @@
         <v>16</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
     </row>
     <row r="39" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -889,7 +922,7 @@
         <v>16</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
     </row>
     <row r="40" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -900,13 +933,13 @@
         <v>6</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E40" s="3" t="s">
         <v>16</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
quebrei o epico HU1
</commit_message>
<xml_diff>
--- a/Close Care/(excel) Ordem de prioridade.xlsx
+++ b/Close Care/(excel) Ordem de prioridade.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\uniflgoncalves\Documents\GitHub\CloseCare-GEST.PROJ.SOFT\Close Care\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FECA6CBB-A5D7-4880-B9AE-27675E53EA1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ADDF26D-4163-47D2-8561-00642CC02322}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4B4DFAF-313B-4775-A4C5-2B6A73696C89}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="48">
   <si>
     <t>ID</t>
   </si>
@@ -165,6 +165,37 @@
   <si>
     <t>Como paciente com falta de mobilidade ou profissional, quero realizar login digitando minhas credenciais no aplicativo 
 para acessar minha conta e utilizar as funcionalidades disponíveis da plataforma.</t>
+  </si>
+  <si>
+    <t>Como paciente com mobilidade reduzida ou idoso, quero selecionar o tipo de profissional de saúde 
+para atendimento domiciliar para encontrar o atendimento adequado.</t>
+  </si>
+  <si>
+    <t>Como paciente, quero visualizar as datas e horários disponíveis do profissional escolhido para escolher um horário livre.</t>
+  </si>
+  <si>
+    <t>Como paciente, quero confirmar o agendamento da consulta domiciliar para garantir minha reserva.</t>
+  </si>
+  <si>
+    <t>Como paciente, quero ser informado quando um horário já estiver ocupado para escolher outra opção.</t>
+  </si>
+  <si>
+    <t>Como paciente, quero utilizar meu endereço cadastrado no agendamento para que o atendimento seja realizado no local correto.</t>
+  </si>
+  <si>
+    <t>Épico:</t>
+  </si>
+  <si>
+    <t>HU16</t>
+  </si>
+  <si>
+    <t>HU17</t>
+  </si>
+  <si>
+    <t>HU15</t>
+  </si>
+  <si>
+    <t>HU14</t>
   </si>
 </sst>
 </file>
@@ -212,7 +243,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -220,11 +251,63 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="7"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="7"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="7"/>
+      </left>
+      <right style="thin">
+        <color theme="7"/>
+      </right>
+      <top style="thin">
+        <color theme="7"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="7"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="7"/>
+      </top>
+      <bottom style="thin">
+        <color theme="7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="7"/>
+      </left>
+      <right style="thin">
+        <color theme="7"/>
+      </right>
+      <top style="thin">
+        <color theme="7"/>
+      </top>
+      <bottom style="thin">
+        <color theme="7"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -248,6 +331,30 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -284,8 +391,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4289C8F6-47EF-48A8-9D30-E2FC98F94D0A}" name="Tabela1" displayName="Tabela1" ref="B2:E15" headerRowDxfId="4">
-  <autoFilter ref="B2:E15" xr:uid="{4289C8F6-47EF-48A8-9D30-E2FC98F94D0A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4289C8F6-47EF-48A8-9D30-E2FC98F94D0A}" name="Tabela1" displayName="Tabela1" ref="B2:E19" headerRowDxfId="4">
+  <autoFilter ref="B2:E19" xr:uid="{4289C8F6-47EF-48A8-9D30-E2FC98F94D0A}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{985DA469-90E4-4E24-8BE5-72DD8AC4D4B7}" name="Prioridade" totalsRowLabel="Total" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{8CF543ED-69A6-4089-B1C8-916B531B30CB}" name="ID" dataDxfId="2"/>
@@ -613,12 +720,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3D1F92C-1AF3-4A95-B439-F4557C2C0F00}">
-  <dimension ref="B2:F40"/>
+  <dimension ref="B2:F39"/>
   <sheetFormatPr defaultRowHeight="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="11.7109375" customWidth="1"/>
     <col min="3" max="3" width="8.5703125" customWidth="1"/>
-    <col min="4" max="4" width="123.85546875" customWidth="1"/>
+    <col min="4" max="4" width="131" customWidth="1"/>
     <col min="5" max="5" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -642,7 +749,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="D3" s="8" t="s">
         <v>36</v>
@@ -650,16 +757,14 @@
       <c r="E3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="F3" s="1"/>
     </row>
     <row r="4" spans="2:6" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="5">
         <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="D4" s="8" t="s">
         <v>37</v>
@@ -667,16 +772,14 @@
       <c r="E4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="F4" s="1"/>
     </row>
     <row r="5" spans="2:6" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="5">
         <v>3</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>35</v>
@@ -690,110 +793,104 @@
       <c r="B6" s="5">
         <v>4</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="7" spans="2:6" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D6" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" s="1"/>
+    </row>
+    <row r="7" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="5">
         <v>5</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="D7" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="8" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D7" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" s="1"/>
+    </row>
+    <row r="8" spans="2:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="5">
         <v>6</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="9" spans="2:6" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C8" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" s="1"/>
+    </row>
+    <row r="9" spans="2:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="5">
         <v>7</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="E9" s="3" t="s">
+      <c r="C9" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="E9" s="11" t="s">
         <v>16</v>
       </c>
       <c r="F9" s="1"/>
     </row>
-    <row r="10" spans="2:6" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="5">
         <v>8</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="E10" s="3" t="s">
+      <c r="C10" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="E10" s="15" t="s">
         <v>16</v>
       </c>
       <c r="F10" s="1"/>
     </row>
-    <row r="11" spans="2:6" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:6" ht="45" x14ac:dyDescent="0.25">
       <c r="B11" s="5">
         <v>9</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>16</v>
       </c>
       <c r="F11" s="1"/>
     </row>
-    <row r="12" spans="2:6" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="5">
         <v>10</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D12" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>18</v>
+        <v>10</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>16</v>
       </c>
       <c r="F12" s="1"/>
     </row>
@@ -802,13 +899,13 @@
         <v>11</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>18</v>
+        <v>30</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>16</v>
       </c>
       <c r="F13" s="1"/>
     </row>
@@ -817,13 +914,13 @@
         <v>12</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>18</v>
+        <v>33</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>16</v>
       </c>
       <c r="F14" s="1"/>
     </row>
@@ -832,40 +929,126 @@
         <v>13</v>
       </c>
       <c r="C15" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="5">
+        <v>14</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="5">
+        <v>15</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D17" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="5">
+        <v>16</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="5">
+        <v>17</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D19" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E19" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="F15" s="1"/>
+    </row>
+    <row r="27" spans="2:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="B27" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C27" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="D27" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="E27" s="11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="34" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B34" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F34" s="1"/>
     </row>
     <row r="35" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C35" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="D35" s="6" t="s">
+      <c r="B35" s="5">
         <v>1</v>
       </c>
-      <c r="E35" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="F35" s="1"/>
+      <c r="C35" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="36" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>16</v>
@@ -876,13 +1059,13 @@
     </row>
     <row r="37" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="5">
+        <v>4</v>
+      </c>
+      <c r="C37" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C37" s="1" t="s">
-        <v>21</v>
-      </c>
       <c r="D37" s="2" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="E37" s="3" t="s">
         <v>16</v>
@@ -893,13 +1076,13 @@
     </row>
     <row r="38" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E38" s="3" t="s">
         <v>16</v>
@@ -910,35 +1093,18 @@
     </row>
     <row r="39" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E39" s="3" t="s">
         <v>16</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="40" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="5">
-        <v>6</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E40" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F40" s="1" t="s">
         <v>24</v>
       </c>
     </row>

</xml_diff>